<commit_message>
Dailed in connector positions.
</commit_message>
<xml_diff>
--- a/Project Outputs for Vehicle_Interface_Tester/BOM/Bill of Materials-Vehicle_Interface_Tester.xlsx
+++ b/Project Outputs for Vehicle_Interface_Tester/BOM/Bill of Materials-Vehicle_Interface_Tester.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT_Local\Vehicle_Interface_Tester_PCB\Project Outputs for Vehicle_Interface_Tester\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT_local\Vehicle_Interface_Tester_PCB\Project Outputs for Vehicle_Interface_Tester\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7B1BD69D-1EC0-4FCA-A676-A0A228D7ED80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C1F35956-D3C2-461A-B9F8-6E448297AFE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2280" yWindow="2280" windowWidth="28800" windowHeight="15370" xr2:uid="{A50B204F-1A43-4FFF-9561-E3BDB865937A}"/>
+    <workbookView xWindow="4930" yWindow="5090" windowWidth="37450" windowHeight="11680" xr2:uid="{63A2FF94-0E44-4074-84AD-4B72729AED73}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill of Materials-Vehicle_Inter" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="275">
   <si>
     <t>Designator</t>
   </si>
@@ -351,21 +351,6 @@
     <t>SS56B</t>
   </si>
   <si>
-    <t>F1</t>
-  </si>
-  <si>
-    <t>1.5A 9.73mm Surface Mount Fuse (with Holder) SMD,9.7x5mm, Littlefuse 015401.5DRT</t>
-  </si>
-  <si>
-    <t>C2936103</t>
-  </si>
-  <si>
-    <t>SMD,10.62×3.81mm</t>
-  </si>
-  <si>
-    <t>1.5A</t>
-  </si>
-  <si>
     <t>J1</t>
   </si>
   <si>
@@ -609,7 +594,7 @@
     <t>24.9K</t>
   </si>
   <si>
-    <t>R3, R16, R19</t>
+    <t>R3, R10, R16, R19</t>
   </si>
   <si>
     <t>10K ohm, Resistor, ±1%, 0402 (1005)</t>
@@ -645,19 +630,7 @@
     <t>100K</t>
   </si>
   <si>
-    <t>R6</t>
-  </si>
-  <si>
-    <t>5.1K ohm, 0402 (1005)</t>
-  </si>
-  <si>
-    <t>C482212</t>
-  </si>
-  <si>
-    <t>5.1K</t>
-  </si>
-  <si>
-    <t>R7</t>
+    <t>R6, R7</t>
   </si>
   <si>
     <t>56K ohm, Resistor, ±1%, 0402 (1005)</t>
@@ -681,7 +654,31 @@
     <t>10M</t>
   </si>
   <si>
-    <t>R9, R10, R18</t>
+    <t>R13, R14, R15</t>
+  </si>
+  <si>
+    <t>4.7K ohm, Resistor, ±1%, 0402 (1005)</t>
+  </si>
+  <si>
+    <t>C25900</t>
+  </si>
+  <si>
+    <t>4.7K</t>
+  </si>
+  <si>
+    <t>R17</t>
+  </si>
+  <si>
+    <t>2.2K ohm, Resistor, ±1%, 1/4W, 1206 (3216)</t>
+  </si>
+  <si>
+    <t>C17948</t>
+  </si>
+  <si>
+    <t>2.2K</t>
+  </si>
+  <si>
+    <t>R18</t>
   </si>
   <si>
     <t>1K ohm, Resistor, ±1%, 0402 (1005)</t>
@@ -693,30 +690,6 @@
     <t>1K</t>
   </si>
   <si>
-    <t>R13, R14, R15</t>
-  </si>
-  <si>
-    <t>4.7K ohm, Resistor, ±1%, 0402 (1005)</t>
-  </si>
-  <si>
-    <t>C25900</t>
-  </si>
-  <si>
-    <t>4.7K</t>
-  </si>
-  <si>
-    <t>R17</t>
-  </si>
-  <si>
-    <t>2.2K ohm, Resistor, ±1%, 1/4W, 1206 (3216)</t>
-  </si>
-  <si>
-    <t>C17948</t>
-  </si>
-  <si>
-    <t>2.2K</t>
-  </si>
-  <si>
     <t>R20</t>
   </si>
   <si>
@@ -820,21 +793,6 @@
   </si>
   <si>
     <t>15K</t>
-  </si>
-  <si>
-    <t>SW1</t>
-  </si>
-  <si>
-    <t>Switch, Tactile, 5x2.9mm, Panasonic EVPAA202K</t>
-  </si>
-  <si>
-    <t>C79147</t>
-  </si>
-  <si>
-    <t>SMD-4P,3.5x2.9mm</t>
-  </si>
-  <si>
-    <t>Switch Tac 5x2.9mm</t>
   </si>
   <si>
     <t>U1</t>
@@ -1270,8 +1228,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DADF658-319E-47D6-9434-280B78EE7CD3}">
-  <dimension ref="A1:F65"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7511C9B1-31A7-41E1-9AB0-8FA709560183}">
+  <dimension ref="A1:F62"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="3" width="18.81640625" customWidth="1"/>
@@ -1813,47 +1771,47 @@
         <v>119</v>
       </c>
       <c r="E27" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F27" s="2" t="s">
         <v>120</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="C28" s="1">
+        <v>2</v>
+      </c>
+      <c r="D28" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C28" s="1">
-        <v>1</v>
-      </c>
-      <c r="D28" s="2" t="s">
+      <c r="E28" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F28" s="2" t="s">
         <v>124</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B29" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="C29" s="1">
+        <v>1</v>
+      </c>
+      <c r="D29" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="C29" s="1">
-        <v>2</v>
-      </c>
-      <c r="D29" s="2" t="s">
+      <c r="E29" s="2" t="s">
         <v>128</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>120</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>129</v>
@@ -1887,7 +1845,7 @@
         <v>136</v>
       </c>
       <c r="C31" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>137</v>
@@ -1907,7 +1865,7 @@
         <v>141</v>
       </c>
       <c r="C32" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>142</v>
@@ -2007,7 +1965,7 @@
         <v>166</v>
       </c>
       <c r="C37" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>167</v>
@@ -2027,7 +1985,7 @@
         <v>171</v>
       </c>
       <c r="C38" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>172</v>
@@ -2073,387 +2031,387 @@
         <v>182</v>
       </c>
       <c r="E40" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F40" s="2" t="s">
         <v>183</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="B41" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="B41" s="2" t="s">
+      <c r="C41" s="1">
+        <v>1</v>
+      </c>
+      <c r="D41" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="C41" s="1">
-        <v>1</v>
-      </c>
-      <c r="D41" s="2" t="s">
+      <c r="E41" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F41" s="2" t="s">
         <v>187</v>
-      </c>
-      <c r="E41" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F41" s="2" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="B42" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="C42" s="1">
+        <v>4</v>
+      </c>
+      <c r="D42" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="C42" s="1">
-        <v>1</v>
-      </c>
-      <c r="D42" s="2" t="s">
+      <c r="E42" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F42" s="2" t="s">
         <v>191</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="B43" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="C43" s="1">
+        <v>1</v>
+      </c>
+      <c r="D43" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="C43" s="1">
-        <v>3</v>
-      </c>
-      <c r="D43" s="2" t="s">
+      <c r="E43" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F43" s="2" t="s">
         <v>195</v>
-      </c>
-      <c r="E43" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="B44" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="C44" s="1">
+        <v>1</v>
+      </c>
+      <c r="D44" s="2" t="s">
         <v>198</v>
-      </c>
-      <c r="C44" s="1">
-        <v>1</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>199</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>9</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="B45" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="B45" s="2" t="s">
+      <c r="C45" s="1">
+        <v>2</v>
+      </c>
+      <c r="D45" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="C45" s="1">
-        <v>1</v>
-      </c>
-      <c r="D45" s="2" t="s">
+      <c r="E45" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F45" s="2" t="s">
         <v>203</v>
-      </c>
-      <c r="E45" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F45" s="2" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="B46" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="C46" s="1">
+        <v>2</v>
+      </c>
+      <c r="D46" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="C46" s="1">
-        <v>1</v>
-      </c>
-      <c r="D46" s="2" t="s">
+      <c r="E46" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F46" s="2" t="s">
         <v>207</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F46" s="2" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="B47" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="B47" s="2" t="s">
+      <c r="C47" s="1">
+        <v>3</v>
+      </c>
+      <c r="D47" s="2" t="s">
         <v>210</v>
-      </c>
-      <c r="C47" s="1">
-        <v>1</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>211</v>
       </c>
       <c r="E47" s="2" t="s">
         <v>24</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="B48" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="B48" s="2" t="s">
+      <c r="C48" s="1">
+        <v>1</v>
+      </c>
+      <c r="D48" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="C48" s="1">
-        <v>2</v>
-      </c>
-      <c r="D48" s="2" t="s">
+      <c r="E48" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F48" s="2" t="s">
         <v>215</v>
-      </c>
-      <c r="E48" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F48" s="2" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="B49" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="B49" s="2" t="s">
+      <c r="C49" s="1">
+        <v>1</v>
+      </c>
+      <c r="D49" s="2" t="s">
         <v>218</v>
-      </c>
-      <c r="C49" s="1">
-        <v>3</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>219</v>
       </c>
       <c r="E49" s="2" t="s">
         <v>24</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="B50" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="B50" s="2" t="s">
+      <c r="C50" s="1">
+        <v>1</v>
+      </c>
+      <c r="D50" s="2" t="s">
         <v>222</v>
-      </c>
-      <c r="C50" s="1">
-        <v>3</v>
-      </c>
-      <c r="D50" s="2" t="s">
-        <v>223</v>
       </c>
       <c r="E50" s="2" t="s">
         <v>24</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>224</v>
+        <v>199</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="C51" s="1">
+        <v>1</v>
+      </c>
+      <c r="D51" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="B51" s="2" t="s">
+      <c r="E51" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F51" s="2" t="s">
         <v>226</v>
-      </c>
-      <c r="C51" s="1">
-        <v>1</v>
-      </c>
-      <c r="D51" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="E51" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F51" s="2" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="C52" s="1">
+        <v>1</v>
+      </c>
+      <c r="D52" s="2" t="s">
         <v>229</v>
-      </c>
-      <c r="B52" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="C52" s="1">
-        <v>1</v>
-      </c>
-      <c r="D52" s="2" t="s">
-        <v>231</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>24</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>204</v>
+        <v>230</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="B53" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="B53" s="2" t="s">
+      <c r="C53" s="1">
+        <v>1</v>
+      </c>
+      <c r="D53" s="2" t="s">
         <v>233</v>
-      </c>
-      <c r="C53" s="1">
-        <v>1</v>
-      </c>
-      <c r="D53" s="2" t="s">
-        <v>234</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>24</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="B54" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="B54" s="2" t="s">
+      <c r="C54" s="1">
+        <v>1</v>
+      </c>
+      <c r="D54" s="2" t="s">
         <v>237</v>
-      </c>
-      <c r="C54" s="1">
-        <v>1</v>
-      </c>
-      <c r="D54" s="2" t="s">
-        <v>238</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>24</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="B55" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="B55" s="2" t="s">
+      <c r="C55" s="1">
+        <v>1</v>
+      </c>
+      <c r="D55" s="2" t="s">
         <v>241</v>
-      </c>
-      <c r="C55" s="1">
-        <v>1</v>
-      </c>
-      <c r="D55" s="2" t="s">
-        <v>242</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>24</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="B56" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="B56" s="2" t="s">
+      <c r="C56" s="1">
+        <v>1</v>
+      </c>
+      <c r="D56" s="2" t="s">
         <v>245</v>
-      </c>
-      <c r="C56" s="1">
-        <v>1</v>
-      </c>
-      <c r="D56" s="2" t="s">
-        <v>246</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>24</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="B57" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="B57" s="2" t="s">
+      <c r="C57" s="1">
+        <v>1</v>
+      </c>
+      <c r="D57" s="2" t="s">
         <v>249</v>
-      </c>
-      <c r="C57" s="1">
-        <v>1</v>
-      </c>
-      <c r="D57" s="2" t="s">
-        <v>250</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>24</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="B58" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="B58" s="2" t="s">
+      <c r="C58" s="1">
+        <v>1</v>
+      </c>
+      <c r="D58" s="2" t="s">
         <v>253</v>
-      </c>
-      <c r="C58" s="1">
-        <v>1</v>
-      </c>
-      <c r="D58" s="2" t="s">
-        <v>254</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>24</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="B59" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="B59" s="2" t="s">
+      <c r="C59" s="1">
+        <v>1</v>
+      </c>
+      <c r="D59" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="C59" s="1">
-        <v>1</v>
-      </c>
-      <c r="D59" s="2" t="s">
+      <c r="E59" s="2" t="s">
         <v>258</v>
-      </c>
-      <c r="E59" s="2" t="s">
-        <v>24</v>
       </c>
       <c r="F59" s="2" t="s">
         <v>259</v>
@@ -2473,110 +2431,50 @@
         <v>262</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>24</v>
+        <v>263</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C61" s="1">
         <v>1</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C62" s="1">
         <v>1</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A63" s="2" t="s">
         <v>274</v>
-      </c>
-      <c r="B63" s="2" t="s">
-        <v>275</v>
-      </c>
-      <c r="C63" s="1">
-        <v>1</v>
-      </c>
-      <c r="D63" s="2" t="s">
-        <v>276</v>
-      </c>
-      <c r="E63" s="2" t="s">
-        <v>277</v>
-      </c>
-      <c r="F63" s="2" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A64" s="2" t="s">
-        <v>279</v>
-      </c>
-      <c r="B64" s="2" t="s">
-        <v>280</v>
-      </c>
-      <c r="C64" s="1">
-        <v>1</v>
-      </c>
-      <c r="D64" s="2" t="s">
-        <v>281</v>
-      </c>
-      <c r="E64" s="2" t="s">
-        <v>282</v>
-      </c>
-      <c r="F64" s="2" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A65" s="2" t="s">
-        <v>284</v>
-      </c>
-      <c r="B65" s="2" t="s">
-        <v>285</v>
-      </c>
-      <c r="C65" s="1">
-        <v>1</v>
-      </c>
-      <c r="D65" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="E65" s="2" t="s">
-        <v>287</v>
-      </c>
-      <c r="F65" s="2" t="s">
-        <v>288</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Worked on component placement alignment with dev board connectors.
</commit_message>
<xml_diff>
--- a/Project Outputs for Vehicle_Interface_Tester/BOM/Bill of Materials-Vehicle_Interface_Tester.xlsx
+++ b/Project Outputs for Vehicle_Interface_Tester/BOM/Bill of Materials-Vehicle_Interface_Tester.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT_local\Vehicle_Interface_Tester_PCB\Project Outputs for Vehicle_Interface_Tester\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C1F35956-D3C2-461A-B9F8-6E448297AFE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9ED0D0F1-F9FA-4BE2-A8AE-94F3C2EAC5BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4930" yWindow="5090" windowWidth="37450" windowHeight="11680" xr2:uid="{63A2FF94-0E44-4074-84AD-4B72729AED73}"/>
+    <workbookView xWindow="0" yWindow="5060" windowWidth="37450" windowHeight="11680" xr2:uid="{CE3CD6AD-04C6-4C04-BF63-6D96B3AD1D3D}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill of Materials-Vehicle_Inter" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="282">
   <si>
     <t>Designator</t>
   </si>
@@ -222,7 +222,7 @@
     <t>22uF</t>
   </si>
   <si>
-    <t>D1, D9</t>
+    <t>D1, D8, D9</t>
   </si>
   <si>
     <t>Schottky Diode, 5A, 30V, SOD-128</t>
@@ -396,7 +396,7 @@
     <t>J4, J5</t>
   </si>
   <si>
-    <t>6 Pos, 1.25mm Pitch, Horizontal SMD</t>
+    <t>6 Pos, 1.25mm Pitch, PicoBlade, Horizontal SMD</t>
   </si>
   <si>
     <t>C17393620</t>
@@ -435,6 +435,18 @@
     <t>USB4800-03-A</t>
   </si>
   <si>
+    <t>J8</t>
+  </si>
+  <si>
+    <t>JTAG 14 Pos Header, 1.27mm Pitch, (.5"), (ST Micro)</t>
+  </si>
+  <si>
+    <t>C17540447</t>
+  </si>
+  <si>
+    <t>JTAG 14 Pos Header 1.27mm Pitch (.5") (ST Micro)</t>
+  </si>
+  <si>
     <t>J10, J11</t>
   </si>
   <si>
@@ -654,6 +666,18 @@
     <t>10M</t>
   </si>
   <si>
+    <t>R11, R12</t>
+  </si>
+  <si>
+    <t>2K ohm, ±1%, 0603 (1608)</t>
+  </si>
+  <si>
+    <t>C22975</t>
+  </si>
+  <si>
+    <t>2K</t>
+  </si>
+  <si>
     <t>R13, R14, R15</t>
   </si>
   <si>
@@ -730,9 +754,6 @@
   </si>
   <si>
     <t>C4109</t>
-  </si>
-  <si>
-    <t>2K</t>
   </si>
   <si>
     <t>R25</t>
@@ -1228,8 +1249,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7511C9B1-31A7-41E1-9AB0-8FA709560183}">
-  <dimension ref="A1:F62"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C6A631F-4C32-451B-969A-2B90658A9F3F}">
+  <dimension ref="A1:F64"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="3" width="18.81640625" customWidth="1"/>
@@ -1545,7 +1566,7 @@
         <v>65</v>
       </c>
       <c r="C16" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>66</v>
@@ -1845,193 +1866,193 @@
         <v>136</v>
       </c>
       <c r="C31" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>137</v>
       </c>
       <c r="E31" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="F31" s="2" t="s">
         <v>138</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="C32" s="1">
+        <v>2</v>
+      </c>
+      <c r="D32" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="C32" s="1">
-        <v>1</v>
-      </c>
-      <c r="D32" s="2" t="s">
+      <c r="E32" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="E32" s="2" t="s">
+      <c r="F32" s="2" t="s">
         <v>143</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B33" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="C33" s="1">
+        <v>1</v>
+      </c>
+      <c r="D33" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="C33" s="1">
-        <v>1</v>
-      </c>
-      <c r="D33" s="2" t="s">
+      <c r="E33" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="E33" s="2" t="s">
+      <c r="F33" s="2" t="s">
         <v>148</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B34" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="C34" s="1">
+        <v>1</v>
+      </c>
+      <c r="D34" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="C34" s="1">
-        <v>1</v>
-      </c>
-      <c r="D34" s="2" t="s">
+      <c r="E34" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="E34" s="2" t="s">
+      <c r="F34" s="2" t="s">
         <v>153</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B35" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="C35" s="1">
+        <v>1</v>
+      </c>
+      <c r="D35" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="C35" s="1">
-        <v>1</v>
-      </c>
-      <c r="D35" s="2" t="s">
+      <c r="E35" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="E35" s="2" t="s">
+      <c r="F35" s="2" t="s">
         <v>158</v>
-      </c>
-      <c r="F35" s="2" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="B36" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="C36" s="1">
+        <v>1</v>
+      </c>
+      <c r="D36" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="C36" s="1">
-        <v>1</v>
-      </c>
-      <c r="D36" s="2" t="s">
+      <c r="E36" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="E36" s="2" t="s">
+      <c r="F36" s="2" t="s">
         <v>163</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="B37" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="C37" s="1">
+        <v>1</v>
+      </c>
+      <c r="D37" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="C37" s="1">
-        <v>2</v>
-      </c>
-      <c r="D37" s="2" t="s">
+      <c r="E37" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="E37" s="2" t="s">
+      <c r="F37" s="2" t="s">
         <v>168</v>
-      </c>
-      <c r="F37" s="2" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="B38" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="C38" s="1">
+        <v>2</v>
+      </c>
+      <c r="D38" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="C38" s="1">
-        <v>1</v>
-      </c>
-      <c r="D38" s="2" t="s">
+      <c r="E38" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="E38" s="2" t="s">
+      <c r="F38" s="2" t="s">
         <v>173</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="B39" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="B39" s="2" t="s">
+      <c r="C39" s="1">
+        <v>1</v>
+      </c>
+      <c r="D39" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="C39" s="1">
-        <v>1</v>
-      </c>
-      <c r="D39" s="2" t="s">
+      <c r="E39" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="E39" s="2" t="s">
+      <c r="F39" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="F39" s="2" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="B40" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="C40" s="1">
+        <v>1</v>
+      </c>
+      <c r="D40" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="C40" s="1">
-        <v>1</v>
-      </c>
-      <c r="D40" s="2" t="s">
+      <c r="E40" s="2" t="s">
         <v>182</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>19</v>
       </c>
       <c r="F40" s="2" t="s">
         <v>183</v>
@@ -2051,7 +2072,7 @@
         <v>186</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="F41" s="2" t="s">
         <v>187</v>
@@ -2065,13 +2086,13 @@
         <v>189</v>
       </c>
       <c r="C42" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>190</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="F42" s="2" t="s">
         <v>191</v>
@@ -2085,13 +2106,13 @@
         <v>193</v>
       </c>
       <c r="C43" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>194</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="F43" s="2" t="s">
         <v>195</v>
@@ -2125,13 +2146,13 @@
         <v>201</v>
       </c>
       <c r="C45" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>202</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="F45" s="2" t="s">
         <v>203</v>
@@ -2151,7 +2172,7 @@
         <v>206</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F46" s="2" t="s">
         <v>207</v>
@@ -2165,13 +2186,13 @@
         <v>209</v>
       </c>
       <c r="C47" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>210</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F47" s="2" t="s">
         <v>211</v>
@@ -2185,13 +2206,13 @@
         <v>213</v>
       </c>
       <c r="C48" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>214</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="F48" s="2" t="s">
         <v>215</v>
@@ -2205,7 +2226,7 @@
         <v>217</v>
       </c>
       <c r="C49" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>218</v>
@@ -2231,50 +2252,50 @@
         <v>222</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>199</v>
+        <v>223</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C51" s="1">
         <v>1</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E51" s="2" t="s">
         <v>24</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C52" s="1">
         <v>1</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>24</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>230</v>
+        <v>203</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.35">
@@ -2334,147 +2355,187 @@
         <v>24</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>242</v>
+        <v>215</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="B56" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="B56" s="2" t="s">
+      <c r="C56" s="1">
+        <v>1</v>
+      </c>
+      <c r="D56" s="2" t="s">
         <v>244</v>
-      </c>
-      <c r="C56" s="1">
-        <v>1</v>
-      </c>
-      <c r="D56" s="2" t="s">
-        <v>245</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>24</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="B57" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="B57" s="2" t="s">
+      <c r="C57" s="1">
+        <v>1</v>
+      </c>
+      <c r="D57" s="2" t="s">
         <v>248</v>
-      </c>
-      <c r="C57" s="1">
-        <v>1</v>
-      </c>
-      <c r="D57" s="2" t="s">
-        <v>249</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>24</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="B58" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="B58" s="2" t="s">
+      <c r="C58" s="1">
+        <v>1</v>
+      </c>
+      <c r="D58" s="2" t="s">
         <v>252</v>
-      </c>
-      <c r="C58" s="1">
-        <v>1</v>
-      </c>
-      <c r="D58" s="2" t="s">
-        <v>253</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>24</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="B59" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="B59" s="2" t="s">
+      <c r="C59" s="1">
+        <v>1</v>
+      </c>
+      <c r="D59" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="C59" s="1">
-        <v>1</v>
-      </c>
-      <c r="D59" s="2" t="s">
+      <c r="E59" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F59" s="2" t="s">
         <v>257</v>
-      </c>
-      <c r="E59" s="2" t="s">
-        <v>258</v>
-      </c>
-      <c r="F59" s="2" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C60" s="1">
+        <v>1</v>
+      </c>
+      <c r="D60" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="B60" s="2" t="s">
+      <c r="E60" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F60" s="2" t="s">
         <v>261</v>
-      </c>
-      <c r="C60" s="1">
-        <v>1</v>
-      </c>
-      <c r="D60" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="E60" s="2" t="s">
-        <v>263</v>
-      </c>
-      <c r="F60" s="2" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="C61" s="1">
+        <v>1</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="E61" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="B61" s="2" t="s">
+      <c r="F61" s="2" t="s">
         <v>266</v>
-      </c>
-      <c r="C61" s="1">
-        <v>1</v>
-      </c>
-      <c r="D61" s="2" t="s">
-        <v>267</v>
-      </c>
-      <c r="E61" s="2" t="s">
-        <v>268</v>
-      </c>
-      <c r="F61" s="2" t="s">
-        <v>269</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="C62" s="1">
+        <v>1</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="E62" s="2" t="s">
         <v>270</v>
       </c>
-      <c r="B62" s="2" t="s">
+      <c r="F62" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="C62" s="1">
-        <v>1</v>
-      </c>
-      <c r="D62" s="2" t="s">
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A63" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="E62" s="2" t="s">
+      <c r="B63" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="F62" s="2" t="s">
+      <c r="C63" s="1">
+        <v>1</v>
+      </c>
+      <c r="D63" s="2" t="s">
         <v>274</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A64" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="C64" s="1">
+        <v>1</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="E64" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="F64" s="2" t="s">
+        <v>281</v>
       </c>
     </row>
   </sheetData>

</xml_diff>